<commit_message>
Document d'analyse final oublié commit
</commit_message>
<xml_diff>
--- a/Mandat 1 - Planification/BelleVibe MatricePermissions.xlsx
+++ b/Mandat 1 - Planification/BelleVibe MatricePermissions.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmaisonneuveqcca-my.sharepoint.com/personal/e6302453_cmaisonneuve_qc_ca/Documents/Session 4/Projet 2/BelleVibe/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_DE1BCBCCDAD57945D02AE09552928C776C0C3DF9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{391B1EBC-7DCD-4540-8A6C-D4823147CBB3}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
@@ -22,92 +27,89 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="26">
   <si>
-    <t xml:space="preserve">Employés</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Superviseur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clients</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permissions standard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seul les superviseurs et les admins peuvent voir les autres employés. Les admins peuvent modifier le statut/position d'un employé (passer de simple employé à superviseur ex). Les superviseurs peuvent modifier les autres infos (ex, changement d'adresse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comptes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historique des dossiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La table "historique des dossiers" se rempli automatiquement dès qu'une action est faite partout dans le système. Seul les superviseurs et admins ont accès à sa lecture mais aucune modification, écriture ou suppréssion est possible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dossiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seul les admins peuvent supprimer des notes, puisqu'elles servent seulement à garder des commentaires ou des remarques sur les clients donc il serait très rare de devoir les supprimer en tant que superviseur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demandes</t>
+    <t>Employés</t>
+  </si>
+  <si>
+    <t>Superviseur</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Clients</t>
+  </si>
+  <si>
+    <t>Read</t>
+  </si>
+  <si>
+    <t>✓</t>
+  </si>
+  <si>
+    <t>Permissions standard</t>
+  </si>
+  <si>
+    <t>Write</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Delete</t>
+  </si>
+  <si>
+    <t>Seul les superviseurs et les admins peuvent voir les autres employés. Les admins peuvent modifier le statut/position d'un employé (passer de simple employé à superviseur ex). Les superviseurs peuvent modifier les autres infos (ex, changement d'adresse)</t>
+  </si>
+  <si>
+    <t>Comptes</t>
+  </si>
+  <si>
+    <t>Historique des dossiers</t>
+  </si>
+  <si>
+    <t>La table "historique des dossiers" se rempli automatiquement dès qu'une action est faite partout dans le système. Seul les superviseurs et admins ont accès à sa lecture mais aucune modification, écriture ou suppréssion est possible.</t>
+  </si>
+  <si>
+    <t>Dossiers</t>
+  </si>
+  <si>
+    <t>Seul les admins peuvent supprimer des notes, puisqu'elles servent seulement à garder des commentaires ou des remarques sur les clients donc il serait très rare de devoir les supprimer en tant que superviseur</t>
+  </si>
+  <si>
+    <t>Demandes</t>
   </si>
   <si>
     <t xml:space="preserve">Les employés devraient seulement écrire et lire les demandes que les clients leur font parvenir. Si on doit en modifier une (ex, l'état de la demande) un superviseur s'en charge. </t>
   </si>
   <si>
-    <t xml:space="preserve">Documents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forfait Dossier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lorsqu’un client appèle, on veut que l’employé puisse voir les forfaits déjà à son dossier, ajouter un nouveau forfait, modifier les forfaits en cours, ou même supprimer un forfait du dossier du client sans avoir à avoir affaire avec un superviseur ou un admin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forfaits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les employés et les superviseurs peuvent voir les forfaits disponnibles mais seul un admin devrait avoir le droit de modifier, supprimer ou créer de nouveaux forfaits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Services</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les employés et les superviseurs peuvent voir les services mais seul un admin devrait avoir d’autres droit sur cette table.</t>
+    <t>Documents</t>
+  </si>
+  <si>
+    <t>Forfait Dossier</t>
+  </si>
+  <si>
+    <t>Lorsqu’un client appèle, on veut que l’employé puisse voir les forfaits déjà à son dossier, ajouter un nouveau forfait, modifier les forfaits en cours, ou même supprimer un forfait du dossier du client sans avoir à avoir affaire avec un superviseur ou un admin.</t>
+  </si>
+  <si>
+    <t>Forfaits</t>
+  </si>
+  <si>
+    <t>Les employés et les superviseurs peuvent voir les forfaits disponnibles mais seul un admin devrait avoir le droit de modifier, supprimer ou créer de nouveaux forfaits.</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Les employés et les superviseurs peuvent voir les services mais seul un admin devrait avoir d’autres droit sur cette table.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -115,22 +117,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -143,14 +130,14 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="22"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -165,150 +152,129 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -361,44 +327,43 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:XFD45"/>
-  <sheetFormatPr defaultColWidth="10.5703125" defaultRowHeight="28.5" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5703125" defaultRowHeight="28.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="10.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="2" width="11.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="43.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="2" width="10.57"/>
+    <col min="1" max="1" width="16.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="4"/>
+    <col min="3" max="5" width="11.7109375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="43.28515625" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="10.5703125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="4" t="s">
+    <row r="1" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="N1" s="3"/>
+    </row>
+    <row r="2" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="6" t="s">
@@ -410,15 +375,15 @@
       <c r="E2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
     </row>
-    <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="4" t="s">
+    <row r="3" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -430,11 +395,11 @@
       <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="4" t="s">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="6" t="s">
@@ -446,11 +411,11 @@
       <c r="E4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="4" t="s">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2"/>
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="6"/>
@@ -460,13 +425,13 @@
       <c r="E5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="6"/>
@@ -476,13 +441,13 @@
       <c r="E6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="4" t="s">
+    <row r="7" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2"/>
+      <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="6"/>
@@ -492,11 +457,11 @@
       <c r="E7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="4" t="s">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2"/>
+      <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="6"/>
@@ -506,11 +471,11 @@
       <c r="E8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="4" t="s">
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C9" s="6"/>
@@ -518,13 +483,13 @@
       <c r="E9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -536,13 +501,13 @@
       <c r="E10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="4" t="s">
+    <row r="11" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2"/>
+      <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="6" t="s">
@@ -554,11 +519,11 @@
       <c r="E11" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="4" t="s">
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2"/>
+      <c r="B12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -570,11 +535,11 @@
       <c r="E12" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="4" t="s">
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C13" s="6"/>
@@ -584,13 +549,13 @@
       <c r="E13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="6"/>
@@ -600,45 +565,45 @@
       <c r="E14" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="4" t="s">
+    <row r="15" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="4" t="s">
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="4" t="s">
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2"/>
+      <c r="B17" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="6" t="s">
@@ -650,13 +615,13 @@
       <c r="E18" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="4" t="s">
+    <row r="19" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="2"/>
+      <c r="B19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="6" t="s">
@@ -668,11 +633,11 @@
       <c r="E19" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="4" t="s">
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="2"/>
+      <c r="B20" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -684,12 +649,12 @@
       <c r="E20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="4"/>
+      <c r="F20" s="1"/>
       <c r="XFD20" s="6"/>
     </row>
-    <row r="21" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="4" t="s">
+    <row r="21" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="2"/>
+      <c r="B21" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="6"/>
@@ -699,13 +664,13 @@
       <c r="E21" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="4"/>
-    </row>
-    <row r="22" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C22" s="6" t="s">
@@ -717,13 +682,13 @@
       <c r="E22" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="4" t="s">
+    <row r="23" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="2"/>
+      <c r="B23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="6" t="s">
@@ -735,11 +700,11 @@
       <c r="E23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="4" t="s">
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2"/>
+      <c r="B24" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C24" s="6" t="s">
@@ -751,11 +716,11 @@
       <c r="E24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="5"/>
-    </row>
-    <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="4" t="s">
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2"/>
+      <c r="B25" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="6"/>
@@ -763,13 +728,13 @@
       <c r="E25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="5"/>
-    </row>
-    <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -781,13 +746,13 @@
       <c r="E26" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5"/>
-      <c r="B27" s="4" t="s">
+    <row r="27" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2"/>
+      <c r="B27" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -799,11 +764,11 @@
       <c r="E27" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5"/>
-      <c r="B28" s="4" t="s">
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2"/>
+      <c r="B28" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="6"/>
@@ -813,11 +778,11 @@
       <c r="E28" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F28" s="5"/>
-    </row>
-    <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5"/>
-      <c r="B29" s="4" t="s">
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2"/>
+      <c r="B29" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C29" s="6"/>
@@ -827,13 +792,13 @@
       <c r="E29" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C30" s="6" t="s">
@@ -845,13 +810,13 @@
       <c r="E30" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5"/>
-      <c r="B31" s="4" t="s">
+    <row r="31" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2"/>
+      <c r="B31" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C31" s="6" t="s">
@@ -863,11 +828,11 @@
       <c r="E31" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F31" s="4"/>
-    </row>
-    <row r="32" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5"/>
-      <c r="B32" s="4" t="s">
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6 16384:16384" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2"/>
+      <c r="B32" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C32" s="6" t="s">
@@ -879,11 +844,11 @@
       <c r="E32" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F32" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5"/>
-      <c r="B33" s="4" t="s">
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="2"/>
+      <c r="B33" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C33" s="6"/>
@@ -893,13 +858,13 @@
       <c r="E33" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C34" s="9" t="s">
@@ -911,13 +876,13 @@
       <c r="E34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5"/>
-      <c r="B35" s="4" t="s">
+    <row r="35" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="2"/>
+      <c r="B35" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C35" s="9" t="s">
@@ -929,11 +894,11 @@
       <c r="E35" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5"/>
-      <c r="B36" s="4" t="s">
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2"/>
+      <c r="B36" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="9" t="s">
@@ -945,11 +910,11 @@
       <c r="E36" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F36" s="5"/>
-    </row>
-    <row r="37" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5"/>
-      <c r="B37" s="4" t="s">
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="2"/>
+      <c r="B37" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C37" s="9" t="s">
@@ -961,13 +926,13 @@
       <c r="E37" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F37" s="5"/>
-    </row>
-    <row r="38" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C38" s="9" t="s">
@@ -979,13 +944,13 @@
       <c r="E38" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5"/>
-      <c r="B39" s="4" t="s">
+    <row r="39" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="2"/>
+      <c r="B39" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C39" s="6"/>
@@ -993,11 +958,11 @@
       <c r="E39" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F39" s="5"/>
-    </row>
-    <row r="40" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5"/>
-      <c r="B40" s="4" t="s">
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2"/>
+      <c r="B40" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C40" s="6"/>
@@ -1005,11 +970,11 @@
       <c r="E40" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5"/>
-      <c r="B41" s="4" t="s">
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="2"/>
+      <c r="B41" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C41" s="6"/>
@@ -1017,13 +982,13 @@
       <c r="E41" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F41" s="5"/>
-    </row>
-    <row r="42" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C42" s="9" t="s">
@@ -1035,13 +1000,13 @@
       <c r="E42" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5"/>
-      <c r="B43" s="4" t="s">
+    <row r="43" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="B43" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="6"/>
@@ -1049,11 +1014,11 @@
       <c r="E43" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F43" s="5"/>
-    </row>
-    <row r="44" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5"/>
-      <c r="B44" s="4" t="s">
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="2"/>
+      <c r="B44" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C44" s="6"/>
@@ -1061,11 +1026,11 @@
       <c r="E44" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F44" s="5"/>
-    </row>
-    <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5"/>
-      <c r="B45" s="4" t="s">
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="2"/>
+      <c r="B45" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C45" s="6"/>
@@ -1073,37 +1038,36 @@
       <c r="E45" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F45" s="5"/>
+      <c r="F45" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="F22:F25"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="F2:F5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="F6:F9"/>
     <mergeCell ref="A10:A13"/>
     <mergeCell ref="F10:F13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="F42:F45"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>

</xml_diff>